<commit_message>
Refine confinement scaling validation
</commit_message>
<xml_diff>
--- a/workflow/automatic_pipeline_3_data_summary/core_profiles_history.xlsx
+++ b/workflow/automatic_pipeline_3_data_summary/core_profiles_history.xlsx
@@ -540,7 +540,7 @@
         <v>0.002936629795628191</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0001178730021923424</v>
+        <v>0.0001280574221734683</v>
       </c>
       <c r="L2" t="n">
         <v>0.5010460022301553</v>
@@ -596,7 +596,7 @@
         <v>0.004702777309924523</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0003414458056757228</v>
+        <v>0.0003292787452511832</v>
       </c>
       <c r="L3" t="n">
         <v>0.9421854789613615</v>
@@ -652,7 +652,7 @@
         <v>0.005296223155629565</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0003076521598217959</v>
+        <v>0.000320114661099256</v>
       </c>
       <c r="L4" t="n">
         <v>0.7861403937161804</v>
@@ -708,7 +708,7 @@
         <v>0.005863312260815866</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0005268562202556927</v>
+        <v>0.0004748978292870822</v>
       </c>
       <c r="L5" t="n">
         <v>1.486591796748295</v>
@@ -764,7 +764,7 @@
         <v>0.006925304657094958</v>
       </c>
       <c r="K6" t="n">
-        <v>0.000230837514166841</v>
+        <v>0.0003010118505928522</v>
       </c>
       <c r="L6" t="n">
         <v>0.08656338033548101</v>
@@ -820,7 +820,7 @@
         <v>0.007169237597271477</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0002384175072130745</v>
+        <v>0.0003220289524798876</v>
       </c>
       <c r="L7" t="n">
         <v>0.1118655433540207</v>
@@ -876,7 +876,7 @@
         <v>0.006064322691210303</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0001130049373188491</v>
+        <v>0.0001896272184274582</v>
       </c>
       <c r="L8" t="n">
         <v>0.0818067427747094</v>
@@ -932,7 +932,7 @@
         <v>0.005156250672661717</v>
       </c>
       <c r="K9" t="n">
-        <v>8.565813497050191e-05</v>
+        <v>0.0001291680743579882</v>
       </c>
       <c r="L9" t="n">
         <v>0.0748831346418713</v>
@@ -988,7 +988,7 @@
         <v>0.007340922348278447</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0001812573607912391</v>
+        <v>0.0002475264450091935</v>
       </c>
       <c r="L10" t="n">
         <v>0.1049283214213189</v>
@@ -1044,7 +1044,7 @@
         <v>0.006198315083349109</v>
       </c>
       <c r="K11" t="n">
-        <v>0.000218033555682052</v>
+        <v>0.0002227130863120594</v>
       </c>
       <c r="L11" t="n">
         <v>0.1810542461633111</v>
@@ -1100,7 +1100,7 @@
         <v>0.005958406531052588</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0002029024495733883</v>
+        <v>0.000196581668287566</v>
       </c>
       <c r="L12" t="n">
         <v>0.1834814716150046</v>
@@ -1156,7 +1156,7 @@
         <v>0.006991855047123395</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0002415194206601924</v>
+        <v>0.0002464383833005207</v>
       </c>
       <c r="L13" t="n">
         <v>0.2031417087832703</v>
@@ -1212,7 +1212,7 @@
         <v>0.006502544904249245</v>
       </c>
       <c r="K14" t="n">
-        <v>0.000184905572003111</v>
+        <v>0.0001932086343621909</v>
       </c>
       <c r="L14" t="n">
         <v>0.1831021110352092</v>
@@ -1268,7 +1268,7 @@
         <v>0.002712442546070879</v>
       </c>
       <c r="K15" t="n">
-        <v>8.410963374070332e-05</v>
+        <v>9.841970596293817e-05</v>
       </c>
       <c r="L15" t="n">
         <v>0.4595694281273204</v>
@@ -1324,7 +1324,7 @@
         <v>0.003247201690949174</v>
       </c>
       <c r="K16" t="n">
-        <v>0.00012400021475954</v>
+        <v>0.0001374106215426707</v>
       </c>
       <c r="L16" t="n">
         <v>1.03394319808012</v>
@@ -1380,7 +1380,7 @@
         <v>0.001577954143457956</v>
       </c>
       <c r="K17" t="n">
-        <v>6.721381229765001e-05</v>
+        <v>6.737962276248998e-05</v>
       </c>
       <c r="L17" t="n">
         <v>1.16238882934574</v>
@@ -1436,7 +1436,7 @@
         <v>0.003023174690136046</v>
       </c>
       <c r="K18" t="n">
-        <v>0.000196058208370557</v>
+        <v>0.0002084523933870434</v>
       </c>
       <c r="L18" t="n">
         <v>1.645516674600572</v>
@@ -1492,7 +1492,7 @@
         <v>0.003721338848469614</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0002817774029192092</v>
+        <v>0.0003231328192949535</v>
       </c>
       <c r="L19" t="n">
         <v>0.7693932328907876</v>
@@ -1548,7 +1548,7 @@
         <v>0.00322539363846682</v>
       </c>
       <c r="K20" t="n">
-        <v>0.0001840027186620936</v>
+        <v>0.0002150478344826561</v>
       </c>
       <c r="L20" t="n">
         <v>0.8554916243544919</v>
@@ -1604,7 +1604,7 @@
         <v>0.002633429102302945</v>
       </c>
       <c r="K21" t="n">
-        <v>0.0001013911796011026</v>
+        <v>0.0001110901435523635</v>
       </c>
       <c r="L21" t="n">
         <v>0.6385684603283981</v>
@@ -1660,7 +1660,7 @@
         <v>0.002853376642974337</v>
       </c>
       <c r="K22" t="n">
-        <v>0.0001912742522596998</v>
+        <v>0.0001984557415866859</v>
       </c>
       <c r="L22" t="n">
         <v>1.861221579496393</v>
@@ -1716,7 +1716,7 @@
         <v>0.002515657577257892</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0001473988800176109</v>
+        <v>0.0001534402345111531</v>
       </c>
       <c r="L23" t="n">
         <v>0.7653206592400262</v>
@@ -1772,7 +1772,7 @@
         <v>0.00352719513995711</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0001277131967693421</v>
+        <v>0.0001423489487564727</v>
       </c>
       <c r="L24" t="n">
         <v>0.6952248144226859</v>
@@ -1828,7 +1828,7 @@
         <v>0.0002016049272896538</v>
       </c>
       <c r="K25" t="n">
-        <v>9.849721313165003e-07</v>
+        <v>1.225407476902901e-06</v>
       </c>
       <c r="L25" t="n">
         <v>0.6324582018927268</v>
@@ -1884,7 +1884,7 @@
         <v>0.006303760744319282</v>
       </c>
       <c r="K26" t="n">
-        <v>0.000358874301128516</v>
+        <v>0.0003984662721945865</v>
       </c>
       <c r="L26" t="n">
         <v>0.8509528897752934</v>
@@ -1940,7 +1940,7 @@
         <v>9.135444706466909e-05</v>
       </c>
       <c r="K27" t="n">
-        <v>3.141010375309113e-07</v>
+        <v>3.906973922781498e-07</v>
       </c>
       <c r="L27" t="n">
         <v>0.6290607140123384</v>
@@ -1996,7 +1996,7 @@
         <v>0.004498893857360711</v>
       </c>
       <c r="K28" t="n">
-        <v>0.0001031164975304604</v>
+        <v>0.0001244650043381653</v>
       </c>
       <c r="L28" t="n">
         <v>0.4057941030645783</v>
@@ -2052,7 +2052,7 @@
         <v>0.0002632752848420742</v>
       </c>
       <c r="K29" t="n">
-        <v>1.249142758977272e-06</v>
+        <v>1.467629319782356e-06</v>
       </c>
       <c r="L29" t="n">
         <v>0.3492260293736171</v>
@@ -2108,7 +2108,7 @@
         <v>9.56311267110035e-05</v>
       </c>
       <c r="K30" t="n">
-        <v>2.243416108966739e-07</v>
+        <v>2.818835083727498e-07</v>
       </c>
       <c r="L30" t="n">
         <v>0.3650942740975447</v>
@@ -2164,7 +2164,7 @@
         <v>8.86413245635293e-05</v>
       </c>
       <c r="K31" t="n">
-        <v>3.455991230202583e-07</v>
+        <v>4.445722178677746e-07</v>
       </c>
       <c r="L31" t="n">
         <v>0.5159032438552223</v>
@@ -2220,7 +2220,7 @@
         <v>0.0006606422871534578</v>
       </c>
       <c r="K32" t="n">
-        <v>7.394887799747538e-06</v>
+        <v>8.843071185332788e-06</v>
       </c>
       <c r="L32" t="n">
         <v>0.4498996814610231</v>
@@ -2276,7 +2276,7 @@
         <v>0.0001927602398238091</v>
       </c>
       <c r="K33" t="n">
-        <v>9.701404044793515e-07</v>
+        <v>1.260197038955387e-06</v>
       </c>
       <c r="L33" t="n">
         <v>0.4609940615377256</v>
@@ -2332,7 +2332,7 @@
         <v>0.006466153349770644</v>
       </c>
       <c r="K34" t="n">
-        <v>0.0002945321515693591</v>
+        <v>0.0003164137352086547</v>
       </c>
       <c r="L34" t="n">
         <v>0.8290900570866081</v>
@@ -2388,7 +2388,7 @@
         <v>0.005567592222106488</v>
       </c>
       <c r="K35" t="n">
-        <v>0.0001853270095935036</v>
+        <v>0.0001927098926568096</v>
       </c>
       <c r="L35" t="n">
         <v>0.653577450391624</v>
@@ -2444,7 +2444,7 @@
         <v>0.005919984501145912</v>
       </c>
       <c r="K36" t="n">
-        <v>0.0002080537730633644</v>
+        <v>0.0002240370363446752</v>
       </c>
       <c r="L36" t="n">
         <v>0.5974860642847155</v>
@@ -2500,7 +2500,7 @@
         <v>3.501809115567524e-05</v>
       </c>
       <c r="K37" t="n">
-        <v>1.101946123884149e-07</v>
+        <v>1.219261438980402e-07</v>
       </c>
       <c r="L37" t="n">
         <v>1.033095408282448</v>
@@ -2556,7 +2556,7 @@
         <v>0.0001278049109980766</v>
       </c>
       <c r="K38" t="n">
-        <v>5.827933860256971e-07</v>
+        <v>7.241247257123375e-07</v>
       </c>
       <c r="L38" t="n">
         <v>0.8162641956664914</v>
@@ -2612,7 +2612,7 @@
         <v>0.005263609823313847</v>
       </c>
       <c r="K39" t="n">
-        <v>0.0002341371563611704</v>
+        <v>0.0002915901212901168</v>
       </c>
       <c r="L39" t="n">
         <v>0.4620267173729863</v>
@@ -2668,7 +2668,7 @@
         <v>0.003475425337022338</v>
       </c>
       <c r="K40" t="n">
-        <v>0.0001286919983043481</v>
+        <v>0.0001581838003718418</v>
       </c>
       <c r="L40" t="n">
         <v>0.5343860755269156</v>
@@ -2724,7 +2724,7 @@
         <v>0.004160705956627877</v>
       </c>
       <c r="K41" t="n">
-        <v>0.0001394611845107999</v>
+        <v>0.0001852302966521968</v>
       </c>
       <c r="L41" t="n">
         <v>0.4080583499898831</v>
@@ -2780,7 +2780,7 @@
         <v>0.001874716821066917</v>
       </c>
       <c r="K42" t="n">
-        <v>4.195149058346772e-05</v>
+        <v>4.729221153714035e-05</v>
       </c>
       <c r="L42" t="n">
         <v>1.000070840608421</v>

</xml_diff>